<commit_message>
Fix: Korrektur der Import-Probleme und Treeview-PN-Lookup
- Alle relativen Imports zu absoluten app.* Imports geändert
- Treeview IID vs. Spaltenwerte Problem behoben
- PN wird jetzt korrekt aus values[0] statt aus IID gelesen
- send_managers und send_selected_employees funktionieren wieder
- Vorschau-Funktionen korrigiert
- Einzelversand zeigt wieder Mitarbeitende nach VG-Auswahl an
- SimpleTrackingSystem um get_dashboard_data und update_entry erweitert
</commit_message>
<xml_diff>
--- a/sap_stammdaten/EXPORT.XLSX
+++ b/sap_stammdaten/EXPORT.XLSX
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R11"/>
+  <dimension ref="A1:R12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -576,8 +576,10 @@
       <c r="O2" t="inlineStr"/>
       <c r="P2" t="inlineStr"/>
       <c r="Q2" t="inlineStr"/>
-      <c r="R2" t="n">
-        <v>2</v>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>2.0</t>
+        </is>
       </c>
     </row>
     <row r="3">
@@ -632,8 +634,10 @@
       <c r="O3" t="inlineStr"/>
       <c r="P3" t="inlineStr"/>
       <c r="Q3" t="inlineStr"/>
-      <c r="R3" t="n">
-        <v>1</v>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
       </c>
     </row>
     <row r="4">
@@ -686,8 +690,10 @@
       <c r="O4" t="inlineStr"/>
       <c r="P4" t="inlineStr"/>
       <c r="Q4" t="inlineStr"/>
-      <c r="R4" t="n">
-        <v>1</v>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
       </c>
     </row>
     <row r="5">
@@ -742,7 +748,11 @@
       <c r="O5" t="inlineStr"/>
       <c r="P5" t="inlineStr"/>
       <c r="Q5" t="inlineStr"/>
-      <c r="R5" t="inlineStr"/>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -798,8 +808,10 @@
           <t>Testbewilligung</t>
         </is>
       </c>
-      <c r="R6" t="n">
-        <v>4</v>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>4.0</t>
+        </is>
       </c>
     </row>
     <row r="7">
@@ -852,8 +864,10 @@
       <c r="O7" t="inlineStr"/>
       <c r="P7" t="inlineStr"/>
       <c r="Q7" t="inlineStr"/>
-      <c r="R7" t="n">
-        <v>3</v>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>3.0</t>
+        </is>
       </c>
     </row>
     <row r="8">
@@ -906,8 +920,10 @@
       <c r="O8" t="inlineStr"/>
       <c r="P8" t="inlineStr"/>
       <c r="Q8" t="inlineStr"/>
-      <c r="R8" t="n">
-        <v>1</v>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
       </c>
     </row>
     <row r="9">
@@ -960,8 +976,10 @@
       <c r="O9" t="inlineStr"/>
       <c r="P9" t="inlineStr"/>
       <c r="Q9" t="inlineStr"/>
-      <c r="R9" t="n">
-        <v>4</v>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>4.0</t>
+        </is>
       </c>
     </row>
     <row r="10">
@@ -1016,8 +1034,10 @@
       <c r="O10" t="inlineStr"/>
       <c r="P10" t="inlineStr"/>
       <c r="Q10" t="inlineStr"/>
-      <c r="R10" t="n">
-        <v>1</v>
+      <c r="R10" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
       </c>
     </row>
     <row r="11">
@@ -1070,8 +1090,68 @@
       <c r="O11" t="inlineStr"/>
       <c r="P11" t="inlineStr"/>
       <c r="Q11" t="inlineStr"/>
-      <c r="R11" t="n">
-        <v>3</v>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>3.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>111111</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Rufname1</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Nachname1</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr"/>
+      <c r="E12" t="inlineStr"/>
+      <c r="F12" t="inlineStr"/>
+      <c r="G12" t="n">
+        <v>90</v>
+      </c>
+      <c r="H12" s="2" t="n">
+        <v>43952</v>
+      </c>
+      <c r="I12" s="2" t="n">
+        <v>44043</v>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>abt1</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>Fachleiter/in Finanzen u. QM</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>111117</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>andreas.ulrich@vd.zh.ch</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr"/>
+      <c r="O12" t="inlineStr"/>
+      <c r="P12" t="inlineStr"/>
+      <c r="Q12" t="inlineStr"/>
+      <c r="R12" t="inlineStr">
+        <is>
+          <t>2.0</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>